<commit_message>
chore(data): archive Facility 三期 368版 (含行政小智) + WSMS + index/history 自学习更新
- Facility 三期需求_20260909: 368人天修订版（估算/报价 Excel + analysis + ai-xiaozhi/ 子目录不单独立项）
- 库状态: 14 项目 / 300 feature / 24 模式中 23 有实例
- 含 20260902 归档与 .bak 备份、WSMS_20260902
</commit_message>
<xml_diff>
--- a/data/estimations/Facility 三期需求_20260713/Facility 三期需求估算.xlsx
+++ b/data/estimations/Facility 三期需求_20260713/Facility 三期需求估算.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaoming\workspace\project-effort-estimation\data\estimations\Facility 三期需求_20260713\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView windowWidth="28800" windowHeight="12255"/>
   </bookViews>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="65">
   <si>
     <t>#</t>
   </si>
@@ -113,10 +118,10 @@
     <t>空调，出门证/货梯两项申请合并</t>
   </si>
   <si>
-    <t>申请合并入口；企微推送消息优化；全部事项内容展示优化</t>
-  </si>
-  <si>
-    <t>数据分类合并，审批处理合并</t>
+    <t>申请合并入口；企微推送消息优化；全部事项内容展示优化4</t>
+  </si>
+  <si>
+    <t>数据分类合并，审批处理合并4</t>
   </si>
   <si>
     <t>在场权益</t>
@@ -126,6 +131,15 @@
   </si>
   <si>
     <t>在场权益维护，链接跳转</t>
+  </si>
+  <si>
+    <t>新增openapi 3个</t>
+  </si>
+  <si>
+    <t>Gateway</t>
+  </si>
+  <si>
+    <t>数据从workday关联读取</t>
   </si>
   <si>
     <t>ISO 45001认证</t>
@@ -242,6 +256,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -250,13 +272,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -601,7 +616,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -619,6 +634,43 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -725,19 +777,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -746,7 +798,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -758,34 +810,34 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -870,7 +922,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -881,16 +933,58 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1239,7 +1333,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="5.70833333333333" customWidth="1"/>
@@ -1278,7 +1372,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="27" spans="1:8">
+    <row r="2" spans="1:8">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1288,32 +1382,30 @@
       <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="7">
         <v>5</v>
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" ht="27" spans="1:8">
+    <row r="3" spans="1:8">
       <c r="A3" s="2"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="7">
         <v>2</v>
       </c>
       <c r="H3" s="3" t="s">
@@ -1328,14 +1420,14 @@
       <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="8"/>
       <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="7">
         <v>2</v>
       </c>
       <c r="H4" s="3" t="s">
@@ -1350,14 +1442,14 @@
       <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="8"/>
+      <c r="E5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="7">
         <v>4</v>
       </c>
       <c r="H5" s="3" t="s">
@@ -1368,14 +1460,12 @@
       <c r="A6" s="2"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="D6" s="8"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="7">
         <v>1</v>
       </c>
       <c r="H6" s="3" t="s">
@@ -1390,14 +1480,14 @@
       <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3" t="s">
+      <c r="D7" s="8"/>
+      <c r="E7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="7">
         <v>3</v>
       </c>
       <c r="H7" s="3" t="s">
@@ -1408,14 +1498,12 @@
       <c r="A8" s="2"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="D8" s="8"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="7">
         <v>2</v>
       </c>
       <c r="H8" s="3" t="s">
@@ -1427,161 +1515,151 @@
         <v>5</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3" t="s">
+      <c r="D9" s="8"/>
+      <c r="E9" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="5">
-        <v>4</v>
-      </c>
-      <c r="H9" s="3" t="s">
+      <c r="G9" s="13">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="2"/>
       <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="C10" s="14"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="5">
-        <v>4</v>
-      </c>
-      <c r="H10" s="3" t="s">
+      <c r="G10" s="13">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="2">
+      <c r="A11" s="16">
         <v>6</v>
       </c>
       <c r="B11" s="3"/>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="7">
         <v>2</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" ht="27" spans="1:8">
-      <c r="A12" s="2">
+    <row r="12" spans="1:8">
+      <c r="A12" s="17"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" s="7">
+        <v>2</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" ht="27" spans="1:8">
+      <c r="A13" s="2">
         <v>7</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G13" s="7">
         <v>10</v>
       </c>
-      <c r="H12" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" ht="27" spans="1:8">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="H13" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" ht="27" spans="1:8">
+      <c r="A14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G14" s="7">
         <v>15</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" ht="54" spans="1:8">
-      <c r="A14" s="2">
-        <v>8</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="5">
-        <v>20</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" ht="27" spans="1:8">
-      <c r="A15" s="2"/>
+    <row r="15" ht="54" spans="1:8">
+      <c r="A15" s="2">
+        <v>8</v>
+      </c>
       <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
+      <c r="C15" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="4" t="s">
+      <c r="E15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="7">
+        <v>20</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" ht="27" spans="1:8">
+      <c r="A16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="5">
-        <v>8</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" ht="27" spans="1:8">
-      <c r="A16" s="2">
-        <v>9</v>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="5">
+      <c r="G16" s="7">
         <v>8</v>
       </c>
       <c r="H16" s="3" t="s">
@@ -1589,227 +1667,254 @@
       </c>
     </row>
     <row r="17" ht="27" spans="1:8">
-      <c r="A17" s="2"/>
+      <c r="A17" s="2">
+        <v>9</v>
+      </c>
       <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+      <c r="C17" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" s="4" t="s">
+      <c r="E17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="7">
+        <v>8</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="2"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G18" s="7">
         <v>5</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" ht="27" spans="1:8">
-      <c r="A18" s="2">
-        <v>10</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="5">
-        <v>10</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="19" ht="40.5" spans="1:8">
-      <c r="A19" s="2"/>
+    <row r="19" spans="1:8">
+      <c r="A19" s="2">
+        <v>10</v>
+      </c>
       <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+      <c r="C19" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F19" s="4" t="s">
+      <c r="E19" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="7">
+        <v>10</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" ht="40.5" spans="1:8">
+      <c r="A20" s="2"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G20" s="7">
         <v>20</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="2">
-        <v>11</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="5">
-        <v>10</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="21" ht="27" spans="1:8">
-      <c r="A21" s="2"/>
+    <row r="21" spans="1:8">
+      <c r="A21" s="2">
+        <v>11</v>
+      </c>
       <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
+      <c r="C21" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="D21" s="3"/>
-      <c r="E21" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="4" t="s">
+      <c r="E21" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="7">
+        <v>10</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" ht="27" spans="1:8">
+      <c r="A22" s="2"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G22" s="7">
         <v>12</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="22" ht="27" spans="1:8">
-      <c r="A22" s="2">
-        <v>12</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="5">
-        <v>5</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" ht="27" spans="1:8">
       <c r="A23" s="2">
-        <v>13</v>
-      </c>
-      <c r="B23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="3"/>
+      <c r="E23" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G23" s="5">
-        <f>ROUNDUP(SUM(G2:G21)*0.15,0)</f>
-        <v>23</v>
-      </c>
-      <c r="H23" s="3"/>
+      <c r="F23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="7">
+        <v>5</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
-      <c r="F24" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G24" s="5">
-        <v>5</v>
+      <c r="F24" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G24" s="7">
+        <f>ROUNDUP(SUM(G2:G22)*0.15,0)</f>
+        <v>22</v>
       </c>
       <c r="H24" s="3"/>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G25" s="5">
-        <v>8</v>
+      <c r="F25" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25" s="7">
+        <v>5</v>
       </c>
       <c r="H25" s="3"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
+      <c r="A26" s="2">
+        <v>15</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
       <c r="F26" s="6" t="s">
         <v>61</v>
       </c>
       <c r="G26" s="7">
-        <f>ROUNDUP(SUM(G2:G25),0)</f>
-        <v>188</v>
-      </c>
-      <c r="H26" s="6"/>
+        <v>8</v>
+      </c>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="20"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" s="21">
+        <f>ROUNDUP(SUM(G2:G26),0)</f>
+        <v>181</v>
+      </c>
+      <c r="H27" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="C23:E23"/>
+  <mergeCells count="35">
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B2:B22"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B2:B23"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D2:D11"/>
-    <mergeCell ref="D12:D22"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D2:D12"/>
+    <mergeCell ref="D13:D23"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E21:E22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>